<commit_message>
Fixed DGP I and II. Remade RF and MPBART output for DGP1,2,2* and added the new data with correct class labels.
</commit_message>
<xml_diff>
--- a/output/mpbart_dgp1_output.xlsx
+++ b/output/mpbart_dgp1_output.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5cac48941448979/Bureaublad/msc_thesis/thesis_code/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED800EA1F6F8B8ECE33DB689524EDE9E2BF74" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E205EA8-8D54-403C-BBAE-81571BA7EA38}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED80032A7A7A8386EABBF70B531EDE9E2BF78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9672F35A-FB4D-46CD-ACCA-770152077770}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -378,52 +378,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.255</v>
+        <v>0.188</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.26700000000000002</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.25900000000000001</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.25900000000000001</v>
+        <v>0.19900000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.22800000000000001</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.248</v>
+        <v>0.182</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.247</v>
+        <v>0.19500000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.26200000000000001</v>
+        <v>0.188</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.22800000000000001</v>
+        <v>0.20499999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.24299999999999999</v>
+        <v>0.17599999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -432,7 +432,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.24959999999999999</v>
+        <v>0.189</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -441,7 +441,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>1.3533497535949663E-2</v>
+        <v>1.0370899457402697E-2</v>
       </c>
     </row>
   </sheetData>
@@ -457,52 +457,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.34472406311111098</v>
+        <v>0.27060397866666702</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.36197858844444403</v>
+        <v>0.23983469777777799</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.34864176266666702</v>
+        <v>0.26215417600000002</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.35416633688888899</v>
+        <v>0.29375324800000002</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.32259799022222202</v>
+        <v>0.28696067111111101</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.34546871288888897</v>
+        <v>0.26537082488888902</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.35840810577777799</v>
+        <v>0.28292843288888903</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.35324203466666698</v>
+        <v>0.27746717777777802</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.33161267288888902</v>
+        <v>0.280271725333333</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.34470269511111101</v>
+        <v>0.25607054311111099</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -511,7 +511,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.34655429626666673</v>
+        <v>0.2715415475555556</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -520,7 +520,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>1.1974795254083532E-2</v>
+        <v>1.6137792643821359E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>